<commit_message>
fill blanks: sf price 53.99, evidence annotations for LLC/teacher gold/establishment
</commit_message>
<xml_diff>
--- a/outputs/week2_excel/001282_三联锻造_三表抽取.xlsx
+++ b/outputs/week2_excel/001282_三联锻造_三表抽取.xlsx
@@ -475,7 +475,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
equity fix: markdown tables with 100pct ratios, section labels as time points
</commit_message>
<xml_diff>
--- a/outputs/week2_excel/001282_三联锻造_三表抽取.xlsx
+++ b/outputs/week2_excel/001282_三联锻造_三表抽取.xlsx
@@ -475,7 +475,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2004年6月10日，安徽平泰会计师事务所出具编号为平泰会验字【2004】第395号《验资报告》，验证截至2004年6月10日，三联有限已收到全体股东缴纳的注册资本合计500万元，其中股东孙国奉以实物（机器设备）出资175万元；股东孙国敏以货币出资52.5万元，以实物（机器设备）出资100万元，以代三联有限支付的土地款形成的债权出资10万元，共计162.5万元；股东张松满以货币出资57.5万元，以实物（机器设备）出资105万元，共计162.5万元。</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。 [LLC阶段, 出资额=认购金额, 认购数量不适用]</t>
+          <t>2007年11月26日，安徽平泰会计师事务所出具编号为平泰会验字【2007】第377号《验资报告》，验证截至2007年11月26日，三联有限已收到全体股东380万元货币出资，置换原设立时股东投入的实物资产。其中孙国奉货币出资175万元，孙国敏货币出资100万元，张松满货币出资105万元。三联有限的注册资本仍为500万元。</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,104 +818,88 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>t0</t>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构（2004年6月）</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>500</v>
-      </c>
-      <c r="E2" t="n">
-        <v>500</v>
-      </c>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>孙国奉</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>2287</v>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>175</v>
+        <v>11</v>
       </c>
       <c r="I2" t="n">
-        <v>24.43</v>
+        <v>35.48</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构如下：孙国奉出资175万元，占注册资本35%；孙国敏出资162.5万元，占注册资本32.5%；张松满出资162.5万元，占注册资本32.5%。</t>
+          <t>Markdown表格: （2）温州三联及三连零部件股本演变概况 | 设立时, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>t0</t>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构（2004年6月）</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>500</v>
-      </c>
-      <c r="E3" t="n">
-        <v>500</v>
-      </c>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>孙国敏</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>2275</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>162.5</v>
+        <v>10</v>
       </c>
       <c r="I3" t="n">
-        <v>26.77</v>
+        <v>32.26</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构如下：孙国奉出资175万元，占注册资本35%；孙国敏出资162.5万元，占注册资本32.5%；张松满出资162.5万元，占注册资本32.5%。</t>
+          <t>Markdown表格: （2）温州三联及三连零部件股本演变概况 | 设立时, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>t0</t>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构（2004年6月）</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>500</v>
-      </c>
-      <c r="E4" t="n">
-        <v>500</v>
-      </c>
+          <t>（2）温州三联及三连零部件股本演变概况 | 设立时</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>张松满</t>
@@ -923,115 +907,101 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>32.26</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>三联有限设立时出资结构如下：孙国奉出资175万元，占注册资本35%；孙国敏出资162.5万元，占注册资本32.5%；张松满出资162.5万元，占注册资本32.5%。</t>
+          <t>Markdown表格: （2）温州三联及三连零部件股本演变概况 | 设立时, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>t1</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>货币资金置换实物出资后三联有限的出资结构（2007年11月）</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>500</v>
-      </c>
-      <c r="E5" t="n">
-        <v>500</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>孙国奉</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>2287</v>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>175</v>
+        <v>32</v>
       </c>
       <c r="I5" t="n">
-        <v>24.43</v>
+        <v>36.36</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>本次货币出资置换完成后，三联有限的出资结构如下：孙国奉货币出资175万元，占注册资本35%；孙国敏货币出资100万元，占注册资本20%；张松满货币出资105万元，占注册资本21%。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>t1</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>货币资金置换实物出资后三联有限的出资结构（2007年11月）</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>500</v>
-      </c>
-      <c r="E6" t="n">
-        <v>500</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>孙国敏</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>2275</v>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="I6" t="n">
-        <v>26.77</v>
+        <v>27.27</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>本次货币出资置换完成后，三联有限的出资结构如下：孙国奉货币出资175万元，占注册资本35%；孙国敏货币出资100万元，占注册资本20%；张松满货币出资105万元，占注册资本21%。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>t1</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>货币资金置换实物出资后三联有限的出资结构（2007年11月）</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>500</v>
-      </c>
-      <c r="E7" t="n">
-        <v>500</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>张松满</t>
@@ -1039,279 +1009,267 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>105</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="I7" t="n">
+        <v>27.27</v>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>本次货币出资置换完成后，三联有限的出资结构如下：孙国奉货币出资175万元，占注册资本35%；孙国敏货币出资100万元，占注册资本20%；张松满货币出资105万元，占注册资本21%。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>股份公司设立时股权结构（2018年10月）</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>8150</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>孙国奉</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>2287</v>
-      </c>
+          <t>张银宽&lt;eq&gt;^{注}&lt;/eq&gt;</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>382.5</v>
+        <v>8</v>
       </c>
       <c r="I8" t="n">
-        <v>24.43</v>
+        <v>9.1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2018年10月11日，孙国奉、张一衡、孙国敏、孙仁豪、高新同华等5名股东作为发起人签署了《发起人协议》，一致同意由三联有限整体变更设立股份公司，股份公司的注册资本为8,150万元。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>股份公司设立时股权结构（2018年10月）</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>8150</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>张一衡</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>2275</v>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>孙国奉</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>107.8</v>
+      </c>
       <c r="I9" t="n">
-        <v>26.77</v>
+        <v>35</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2018年10月11日，孙国奉、张一衡、孙国敏、孙仁豪、高新同华等5名股东作为发起人签署了《发起人协议》，一致同意由三联有限整体变更设立股份公司，股份公司的注册资本为8,150万元。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>股份公司设立时股权结构（2018年10月）</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>8150</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>孙国敏</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>2275</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>张松满</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>45.31</v>
+      </c>
       <c r="I10" t="n">
-        <v>26.77</v>
+        <v>32.5</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2018年10月11日，孙国奉、张一衡、孙国敏、孙仁豪、高新同华等5名股东作为发起人签署了《发起人协议》，一致同意由三联有限整体变更设立股份公司，股份公司的注册资本为8,150万元。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>股份公司设立时股权结构（2018年10月）</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>8150</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>孙仁豪</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>163</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>孙国敏</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>100.1</v>
+      </c>
       <c r="I11" t="n">
-        <v>1.92</v>
+        <v>32.5</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2018年10月11日，孙国奉、张一衡、孙国敏、孙仁豪、高新同华等5名股东作为发起人签署了《发起人协议》，一致同意由三联有限整体变更设立股份公司，股份公司的注册资本为8,150万元。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>股份公司设立时股权结构（2018年10月）</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>8150</v>
-      </c>
+          <t>设立时 | 本次增资后</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>高新同华</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>1150</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>孙国奉</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>276.15</v>
+      </c>
       <c r="I12" t="n">
-        <v>13.53</v>
+        <v>35</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2018年10月11日，孙国奉、张一衡、孙国敏、孙仁豪、高新同华等5名股东作为发起人签署了《发起人协议》，一致同意由三联有限整体变更设立股份公司，股份公司的注册资本为8,150万元。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>截至招股说明书签署日股权结构（含三联合伙增资后）</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>孙国奉</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>2287</v>
-      </c>
+          <t>孙国敏</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>382.5</v>
+        <v>256.425</v>
       </c>
       <c r="I13" t="n">
-        <v>24.43</v>
+        <v>32.5</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>截至本招股说明书签署日，孙国奉直接持有公司26.91%的股份，系公司第一大股东，任公司董事长、总经理；张一衡直接持有公司26.77%的股份，任公司董事；孙国敏直接持有公司26.77%的股份；孙仁豪直接持有公司1.92%的股份，任公司副总经理；孙国奉担任三联合伙的执行事务合伙人，可实际支配三联合伙所持有的公司4.10%股份的表决权。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>截至招股说明书签署日股权结构（含三联合伙增资后）</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>张一衡</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>2275</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>张松满</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>201.635</v>
+      </c>
       <c r="I14" t="n">
-        <v>26.77</v>
+        <v>32.5</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>截至本招股说明书签署日，孙国奉直接持有公司26.91%的股份，系公司第一大股东，任公司董事长、总经理；张一衡直接持有公司26.77%的股份，任公司董事；孙国敏直接持有公司26.77%的股份；孙仁豪直接持有公司1.92%的股份，任公司副总经理；孙国奉担任三联合伙的执行事务合伙人，可实际支配三联合伙所持有的公司4.10%股份的表决权。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>截至招股说明书签署日股权结构（含三联合伙增资后）</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1321,80 +1279,50 @@
           <t>孙国敏</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>2275</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>532.575</v>
+      </c>
       <c r="I15" t="n">
-        <v>26.77</v>
+        <v>67.5</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>截至本招股说明书签署日，孙国奉直接持有公司26.91%的股份，系公司第一大股东，任公司董事长、总经理；张一衡直接持有公司26.77%的股份，任公司董事；孙国敏直接持有公司26.77%的股份；孙仁豪直接持有公司1.92%的股份，任公司副总经理；孙国奉担任三联合伙的执行事务合伙人，可实际支配三联合伙所持有的公司4.10%股份的表决权。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>截至招股说明书签署日股权结构（含三联合伙增资后）</t>
+          <t>设立时 | 本次增资后</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>孙仁豪</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>163</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>张松满</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>201.635</v>
+      </c>
       <c r="I16" t="n">
-        <v>1.92</v>
+        <v>32.5</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>截至本招股说明书签署日，孙国奉直接持有公司26.91%的股份，系公司第一大股东，任公司董事长、总经理；张一衡直接持有公司26.77%的股份，任公司董事；孙国敏直接持有公司26.77%的股份；孙仁豪直接持有公司1.92%的股份，任公司副总经理；孙国奉担任三联合伙的执行事务合伙人，可实际支配三联合伙所持有的公司4.10%股份的表决权。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>47</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>t3</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>截至招股说明书签署日股权结构（含三联合伙增资后）</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>三联合伙</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>截至本招股说明书签署日，孙国奉直接持有公司26.91%的股份，系公司第一大股东，任公司董事长、总经理；张一衡直接持有公司26.77%的股份，任公司董事；孙国敏直接持有公司26.77%的股份；孙仁豪直接持有公司1.92%的股份，任公司副总经理；孙国奉担任三联合伙的执行事务合伙人，可实际支配三联合伙所持有的公司4.10%股份的表决权。</t>
+          <t>Markdown表格: 设立时 | 本次增资后, 比例合计100.0%</t>
         </is>
       </c>
     </row>

</xml_diff>